<commit_message>
view mapping and delete all from faculty
</commit_message>
<xml_diff>
--- a/uploads/mapping.xlsx
+++ b/uploads/mapping.xlsx
@@ -26,27 +26,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
-    <t>Faculty ID</t>
-  </si>
-  <si>
-    <t>Student ID</t>
-  </si>
-  <si>
-    <t>FAC66600</t>
-  </si>
-  <si>
-    <t>FAC23400</t>
-  </si>
-  <si>
-    <t>FAC12300</t>
-  </si>
-  <si>
-    <t>Faculty Name</t>
-  </si>
-  <si>
-    <t>Skill ID</t>
-  </si>
-  <si>
     <t>Skill Name</t>
   </si>
   <si>
@@ -84,6 +63,27 @@
   </si>
   <si>
     <t>supra</t>
+  </si>
+  <si>
+    <t>FAC456</t>
+  </si>
+  <si>
+    <t>FAC567</t>
+  </si>
+  <si>
+    <t>FAC678</t>
+  </si>
+  <si>
+    <t>faculty_id</t>
+  </si>
+  <si>
+    <t>faculty_name</t>
+  </si>
+  <si>
+    <t>skill_id</t>
+  </si>
+  <si>
+    <t>student_id</t>
   </si>
 </sst>
 </file>
@@ -443,42 +443,42 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
       <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -486,7 +486,7 @@
         <v>3</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -494,27 +494,27 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E5">
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -522,7 +522,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -530,47 +530,47 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>